<commit_message>
Added new Category for the taxonomy process
</commit_message>
<xml_diff>
--- a/data/raw/category_mapping.xlsx
+++ b/data/raw/category_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DUVAN\Maestria\TFM\transformer-contract-analysis\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F101CF8C-7765-43C5-AA40-2CA35428D972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{004F1B3B-3374-450A-9485-31D4A1F48456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5A2A1962-B33B-44D5-A2FB-CC0C782C3979}"/>
   </bookViews>
@@ -1154,13 +1154,13 @@
         <v>95</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>